<commit_message>
Integrated UDW research results and interactive charts into Laravel dashboard
</commit_message>
<xml_diff>
--- a/results/results_summary.xlsx
+++ b/results/results_summary.xlsx
@@ -23,13 +23,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,37 +435,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>build_time_s</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>total_sources</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>integration_success_pct</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>historical_tracking_pct</t>
         </is>
@@ -471,7 +483,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.08</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
@@ -496,7 +508,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.121</v>
+        <v>0.146</v>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
@@ -521,7 +533,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.098</v>
+        <v>0.127</v>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
@@ -546,7 +558,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.083</v>
+        <v>0.094</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
@@ -574,32 +586,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>query</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>avg_ms</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>min_ms</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>max_ms</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>runs</t>
         </is>
@@ -617,13 +629,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.38</v>
+        <v>0.386</v>
       </c>
       <c r="D2" t="n">
-        <v>0.287</v>
+        <v>0.298</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F2" t="n">
         <v>5</v>
@@ -641,13 +653,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.59</v>
+        <v>0.768</v>
       </c>
       <c r="D3" t="n">
-        <v>0.474</v>
+        <v>0.724</v>
       </c>
       <c r="E3" t="n">
-        <v>0.757</v>
+        <v>0.913</v>
       </c>
       <c r="F3" t="n">
         <v>5</v>
@@ -665,13 +677,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.489</v>
+        <v>0.479</v>
       </c>
       <c r="D4" t="n">
-        <v>0.443</v>
+        <v>0.442</v>
       </c>
       <c r="E4" t="n">
-        <v>0.533</v>
+        <v>0.576</v>
       </c>
       <c r="F4" t="n">
         <v>5</v>
@@ -689,13 +701,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.388</v>
+        <v>0.589</v>
       </c>
       <c r="D5" t="n">
-        <v>0.357</v>
+        <v>0.512</v>
       </c>
       <c r="E5" t="n">
-        <v>0.452</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="F5" t="n">
         <v>5</v>
@@ -713,13 +725,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.332</v>
+        <v>0.326</v>
       </c>
       <c r="D6" t="n">
-        <v>0.284</v>
+        <v>0.297</v>
       </c>
       <c r="E6" t="n">
-        <v>0.427</v>
+        <v>0.382</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
@@ -737,13 +749,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.334</v>
+        <v>0.345</v>
       </c>
       <c r="D7" t="n">
-        <v>0.284</v>
+        <v>0.295</v>
       </c>
       <c r="E7" t="n">
-        <v>0.486</v>
+        <v>0.526</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
@@ -761,13 +773,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.513</v>
+        <v>0.527</v>
       </c>
       <c r="D8" t="n">
-        <v>0.465</v>
+        <v>0.484</v>
       </c>
       <c r="E8" t="n">
-        <v>0.624</v>
+        <v>0.634</v>
       </c>
       <c r="F8" t="n">
         <v>5</v>
@@ -785,13 +797,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.843</v>
+        <v>0.759</v>
       </c>
       <c r="D9" t="n">
-        <v>0.744</v>
+        <v>0.741</v>
       </c>
       <c r="E9" t="n">
-        <v>0.986</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>5</v>
@@ -809,13 +821,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.409</v>
+        <v>0.443</v>
       </c>
       <c r="D10" t="n">
-        <v>0.355</v>
+        <v>0.363</v>
       </c>
       <c r="E10" t="n">
-        <v>0.518</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>5</v>
@@ -833,13 +845,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.295</v>
+        <v>0.479</v>
       </c>
       <c r="D11" t="n">
-        <v>0.284</v>
+        <v>0.457</v>
       </c>
       <c r="E11" t="n">
-        <v>0.324</v>
+        <v>0.53</v>
       </c>
       <c r="F11" t="n">
         <v>5</v>
@@ -857,13 +869,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.371</v>
+        <v>0.36</v>
       </c>
       <c r="D12" t="n">
-        <v>0.305</v>
+        <v>0.3</v>
       </c>
       <c r="E12" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="F12" t="n">
         <v>5</v>
@@ -881,13 +893,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.057</v>
+        <v>1.107</v>
       </c>
       <c r="D13" t="n">
-        <v>0.914</v>
+        <v>1.004</v>
       </c>
       <c r="E13" t="n">
-        <v>1.33</v>
+        <v>1.368</v>
       </c>
       <c r="F13" t="n">
         <v>5</v>
@@ -905,13 +917,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.82</v>
+        <v>0.797</v>
       </c>
       <c r="D14" t="n">
-        <v>0.761</v>
+        <v>0.755</v>
       </c>
       <c r="E14" t="n">
-        <v>0.921</v>
+        <v>0.873</v>
       </c>
       <c r="F14" t="n">
         <v>5</v>
@@ -929,13 +941,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.646</v>
+        <v>0.636</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.546</v>
       </c>
       <c r="E15" t="n">
-        <v>0.86</v>
+        <v>0.847</v>
       </c>
       <c r="F15" t="n">
         <v>5</v>
@@ -953,13 +965,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.34</v>
+        <v>0.306</v>
       </c>
       <c r="D16" t="n">
-        <v>0.284</v>
+        <v>0.294</v>
       </c>
       <c r="E16" t="n">
-        <v>0.432</v>
+        <v>0.344</v>
       </c>
       <c r="F16" t="n">
         <v>5</v>
@@ -977,13 +989,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.394</v>
+        <v>0.358</v>
       </c>
       <c r="D17" t="n">
-        <v>0.296</v>
+        <v>0.303</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.537</v>
       </c>
       <c r="F17" t="n">
         <v>5</v>
@@ -1001,13 +1013,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.378</v>
+        <v>0.391</v>
       </c>
       <c r="D18" t="n">
-        <v>0.36</v>
+        <v>0.369</v>
       </c>
       <c r="E18" t="n">
-        <v>0.403</v>
+        <v>0.433</v>
       </c>
       <c r="F18" t="n">
         <v>5</v>
@@ -1025,13 +1037,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.387</v>
+        <v>0.334</v>
       </c>
       <c r="D19" t="n">
-        <v>0.325</v>
+        <v>0.32</v>
       </c>
       <c r="E19" t="n">
-        <v>0.475</v>
+        <v>0.368</v>
       </c>
       <c r="F19" t="n">
         <v>5</v>
@@ -1049,13 +1061,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.307</v>
+        <v>0.283</v>
       </c>
       <c r="D20" t="n">
-        <v>0.261</v>
+        <v>0.268</v>
       </c>
       <c r="E20" t="n">
-        <v>0.397</v>
+        <v>0.318</v>
       </c>
       <c r="F20" t="n">
         <v>5</v>
@@ -1073,13 +1085,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.153</v>
+        <v>0.124</v>
       </c>
       <c r="D21" t="n">
-        <v>0.137</v>
+        <v>0.112</v>
       </c>
       <c r="E21" t="n">
-        <v>0.201</v>
+        <v>0.149</v>
       </c>
       <c r="F21" t="n">
         <v>5</v>
@@ -1100,12 +1112,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>avg_ms</t>
         </is>
@@ -1118,7 +1130,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6468</v>
+        <v>0.6412</v>
       </c>
     </row>
     <row r="3">
@@ -1128,7 +1140,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4788</v>
+        <v>0.5105999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1138,7 +1150,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4358</v>
+        <v>0.5096000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1148,7 +1160,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3238</v>
+        <v>0.298</v>
       </c>
     </row>
   </sheetData>
@@ -1166,32 +1178,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>new_sources_added</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>total_time_ms</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>avg_time_per_source_ms</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>min_ms</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>max_ms</t>
         </is>
@@ -1300,37 +1312,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>total_rows</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>completeness_pct</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>consistency_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>accuracy_pct</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>dq_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
@@ -1837,34 +1849,34 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>completeness_pct</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>consistency_pct</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>accuracy_pct</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dq_score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Data Vault 2.0</t>
         </is>
@@ -1883,7 +1895,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Inmon 3NF</t>
         </is>
@@ -1902,7 +1914,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Kimball Star Schema</t>
         </is>
@@ -1921,7 +1933,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Unified DW + AI</t>
         </is>
@@ -1954,97 +1966,97 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>anomaly_model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>anomaly_total_samples</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>anomaly_true_anomalies</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>anomaly_predicted_anomalies</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>anomaly_precision_anomaly</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>anomaly_recall_anomaly</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>anomaly_f1_anomaly</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>anomaly_accuracy</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>prediction_model</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>prediction_total_samples</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>prediction_train_size</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>prediction_test_size</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>prediction_accuracy</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prediction_precision_hv</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>prediction_recall_hv</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>prediction_f1_hv</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>prediction_cv_accuracy_mean</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>prediction_cv_accuracy_std</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>prediction_top_feature</t>
         </is>

</xml_diff>